<commit_message>
Updated scripts and data dictionary
</commit_message>
<xml_diff>
--- a/metadata/wash_main_dict.xlsx
+++ b/metadata/wash_main_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Water-Sanitation\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25EB620D-6C40-414C-A827-8E274184CCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2342695A-5E32-4323-8C28-3D671309F4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="781">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="785">
   <si>
     <t>pos</t>
   </si>
@@ -1738,18 +1738,12 @@
     <t>HR09a</t>
   </si>
   <si>
-    <t>In the past six months have you tested positive for any sexually transmitted infections?</t>
-  </si>
-  <si>
     <t>HR09b. If yes, which sexually transmitted infections have you had in the past six months?</t>
   </si>
   <si>
     <t>HR09b</t>
   </si>
   <si>
-    <t>If yes, which sexually transmitted infections have you had in the past six months?</t>
-  </si>
-  <si>
     <t>HR09b. If yes, which sexually transmitted infections have you had in the past six months?/Trichomoniasis</t>
   </si>
   <si>
@@ -1891,9 +1885,6 @@
     <t>HR11</t>
   </si>
   <si>
-    <t>Have ever been screened for cervical cancer?</t>
-  </si>
-  <si>
     <t>HR12. When was your last cervical cancer screening?</t>
   </si>
   <si>
@@ -1909,18 +1900,12 @@
     <t>HR13</t>
   </si>
   <si>
-    <t>What was the results of your last cervical cancer screening?</t>
-  </si>
-  <si>
     <t>HR15. In  the past 1 year  which family  planning method have  you used ?</t>
   </si>
   <si>
     <t>HR15</t>
   </si>
   <si>
-    <t>In  the past 1 year  which family  planning method have  you used ?</t>
-  </si>
-  <si>
     <t>HR15. In  the past 1 year  which family  planning method have  you used ?/Copper IUD</t>
   </si>
   <si>
@@ -2050,9 +2035,6 @@
     <t>WSR01</t>
   </si>
   <si>
-    <t>Are you currently sexually active?</t>
-  </si>
-  <si>
     <t>WSR02. How often do you typically bathe/wash your genital area?</t>
   </si>
   <si>
@@ -2122,18 +2104,12 @@
     <t>WSR05</t>
   </si>
   <si>
-    <t>How many sexual partners have you had in the last two years?</t>
-  </si>
-  <si>
     <t>WQA. How many water samples are available?</t>
   </si>
   <si>
     <t>WQA</t>
   </si>
   <si>
-    <t>How many water samples are available?</t>
-  </si>
-  <si>
     <t>UHPV01. Would you be willing to provide a vaginal swab sample, either through self-collection or with assistance from a trained nurse?</t>
   </si>
   <si>
@@ -2363,6 +2339,42 @@
   </si>
   <si>
     <t>fct</t>
+  </si>
+  <si>
+    <t>Is your primary source of water clean?</t>
+  </si>
+  <si>
+    <t>Currently sexually active</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>Tested positive for any STI past 6 months</t>
+  </si>
+  <si>
+    <t>STI had in the past 6 months</t>
+  </si>
+  <si>
+    <t>Ever been screened for cervical cancer</t>
+  </si>
+  <si>
+    <t>Results of your last cervical cancer screening</t>
+  </si>
+  <si>
+    <t>Family  planning method have  used last 12 months</t>
+  </si>
+  <si>
+    <t>Number of sexual partners had in the last two years</t>
+  </si>
+  <si>
+    <t>Number of water samples available</t>
+  </si>
+  <si>
+    <t>Vaginal swab sample</t>
   </si>
 </sst>
 </file>
@@ -2782,7 +2794,7 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
@@ -2799,7 +2811,7 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
@@ -2816,7 +2828,7 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
@@ -2867,7 +2879,7 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>775</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -2918,7 +2930,7 @@
         <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D12" t="s">
         <v>36</v>
@@ -2952,7 +2964,7 @@
         <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D14" t="s">
         <v>42</v>
@@ -2969,7 +2981,7 @@
         <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D15" t="s">
         <v>45</v>
@@ -2986,7 +2998,7 @@
         <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D16" t="s">
         <v>48</v>
@@ -3003,7 +3015,7 @@
         <v>50</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D17" t="s">
         <v>51</v>
@@ -3054,7 +3066,7 @@
         <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>776</v>
       </c>
       <c r="D20" t="s">
         <v>61</v>
@@ -3071,7 +3083,7 @@
         <v>63</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D21" t="s">
         <v>64</v>
@@ -3088,7 +3100,7 @@
         <v>66</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D22" t="s">
         <v>67</v>
@@ -3105,7 +3117,7 @@
         <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D23" t="s">
         <v>70</v>
@@ -3139,7 +3151,7 @@
         <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D25" t="s">
         <v>76</v>
@@ -3173,7 +3185,7 @@
         <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D27" t="s">
         <v>82</v>
@@ -3292,7 +3304,7 @@
         <v>102</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D34" t="s">
         <v>103</v>
@@ -3326,7 +3338,7 @@
         <v>108</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D36" t="s">
         <v>109</v>
@@ -3360,7 +3372,7 @@
         <v>114</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D38" t="s">
         <v>115</v>
@@ -3377,7 +3389,7 @@
         <v>117</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D39" t="s">
         <v>118</v>
@@ -3394,7 +3406,7 @@
         <v>120</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D40" t="s">
         <v>121</v>
@@ -3411,7 +3423,7 @@
         <v>123</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D41" t="s">
         <v>124</v>
@@ -3428,7 +3440,7 @@
         <v>126</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D42" t="s">
         <v>127</v>
@@ -3445,7 +3457,7 @@
         <v>129</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D43" t="s">
         <v>130</v>
@@ -3462,7 +3474,7 @@
         <v>132</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D44" t="s">
         <v>133</v>
@@ -3479,7 +3491,7 @@
         <v>135</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D45" t="s">
         <v>136</v>
@@ -3496,7 +3508,7 @@
         <v>138</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D46" t="s">
         <v>139</v>
@@ -3513,7 +3525,7 @@
         <v>141</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D47" t="s">
         <v>142</v>
@@ -3530,7 +3542,7 @@
         <v>144</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D48" t="s">
         <v>145</v>
@@ -3564,7 +3576,7 @@
         <v>150</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D50" t="s">
         <v>151</v>
@@ -3581,7 +3593,7 @@
         <v>153</v>
       </c>
       <c r="C51" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D51" t="s">
         <v>154</v>
@@ -3598,7 +3610,7 @@
         <v>156</v>
       </c>
       <c r="C52" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D52" t="s">
         <v>157</v>
@@ -3615,7 +3627,7 @@
         <v>159</v>
       </c>
       <c r="C53" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D53" t="s">
         <v>160</v>
@@ -3632,7 +3644,7 @@
         <v>162</v>
       </c>
       <c r="C54" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D54" t="s">
         <v>163</v>
@@ -3649,7 +3661,7 @@
         <v>165</v>
       </c>
       <c r="C55" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D55" t="s">
         <v>166</v>
@@ -3666,7 +3678,7 @@
         <v>168</v>
       </c>
       <c r="C56" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D56" t="s">
         <v>169</v>
@@ -3683,7 +3695,7 @@
         <v>171</v>
       </c>
       <c r="C57" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D57" t="s">
         <v>172</v>
@@ -3700,7 +3712,7 @@
         <v>174</v>
       </c>
       <c r="C58" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D58" t="s">
         <v>175</v>
@@ -3723,7 +3735,7 @@
         <v>177</v>
       </c>
       <c r="E59" t="s">
-        <v>725</v>
+        <v>717</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
@@ -3734,13 +3746,13 @@
         <v>178</v>
       </c>
       <c r="C60" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D60" t="s">
         <v>179</v>
       </c>
       <c r="E60" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
@@ -3870,7 +3882,7 @@
         <v>200</v>
       </c>
       <c r="C68" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D68" t="s">
         <v>201</v>
@@ -3887,7 +3899,7 @@
         <v>203</v>
       </c>
       <c r="C69" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D69" t="s">
         <v>204</v>
@@ -3904,7 +3916,7 @@
         <v>206</v>
       </c>
       <c r="C70" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D70" t="s">
         <v>207</v>
@@ -3921,7 +3933,7 @@
         <v>209</v>
       </c>
       <c r="C71" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D71" t="s">
         <v>210</v>
@@ -3938,7 +3950,7 @@
         <v>212</v>
       </c>
       <c r="C72" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D72" t="s">
         <v>213</v>
@@ -3955,7 +3967,7 @@
         <v>215</v>
       </c>
       <c r="C73" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D73" t="s">
         <v>216</v>
@@ -3972,7 +3984,7 @@
         <v>218</v>
       </c>
       <c r="C74" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D74" t="s">
         <v>219</v>
@@ -3989,7 +4001,7 @@
         <v>221</v>
       </c>
       <c r="C75" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D75" t="s">
         <v>222</v>
@@ -4023,13 +4035,13 @@
         <v>227</v>
       </c>
       <c r="C77" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D77" t="s">
         <v>228</v>
       </c>
       <c r="E77" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
@@ -4057,7 +4069,7 @@
         <v>232</v>
       </c>
       <c r="C79" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D79" t="s">
         <v>233</v>
@@ -4074,7 +4086,7 @@
         <v>235</v>
       </c>
       <c r="C80" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D80" t="s">
         <v>236</v>
@@ -4097,7 +4109,7 @@
         <v>239</v>
       </c>
       <c r="E81" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
@@ -4108,7 +4120,7 @@
         <v>240</v>
       </c>
       <c r="C82" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D82" t="s">
         <v>241</v>
@@ -4125,7 +4137,7 @@
         <v>243</v>
       </c>
       <c r="C83" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D83" t="s">
         <v>244</v>
@@ -4142,7 +4154,7 @@
         <v>246</v>
       </c>
       <c r="C84" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D84" t="s">
         <v>247</v>
@@ -4176,7 +4188,7 @@
         <v>252</v>
       </c>
       <c r="C86" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D86" t="s">
         <v>253</v>
@@ -4193,7 +4205,7 @@
         <v>255</v>
       </c>
       <c r="C87" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D87" t="s">
         <v>256</v>
@@ -4210,7 +4222,7 @@
         <v>258</v>
       </c>
       <c r="C88" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D88" t="s">
         <v>259</v>
@@ -4227,7 +4239,7 @@
         <v>261</v>
       </c>
       <c r="C89" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D89" t="s">
         <v>262</v>
@@ -4244,7 +4256,7 @@
         <v>264</v>
       </c>
       <c r="C90" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D90" t="s">
         <v>265</v>
@@ -4261,7 +4273,7 @@
         <v>267</v>
       </c>
       <c r="C91" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D91" t="s">
         <v>268</v>
@@ -4295,7 +4307,7 @@
         <v>273</v>
       </c>
       <c r="C93" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D93" t="s">
         <v>274</v>
@@ -4312,7 +4324,7 @@
         <v>276</v>
       </c>
       <c r="C94" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D94" t="s">
         <v>277</v>
@@ -4346,7 +4358,7 @@
         <v>282</v>
       </c>
       <c r="C96" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D96" t="s">
         <v>283</v>
@@ -4363,13 +4375,13 @@
         <v>284</v>
       </c>
       <c r="C97" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D97" t="s">
         <v>285</v>
       </c>
       <c r="E97" t="s">
-        <v>284</v>
+        <v>773</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
@@ -4380,7 +4392,7 @@
         <v>286</v>
       </c>
       <c r="C98" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D98" t="s">
         <v>287</v>
@@ -4397,7 +4409,7 @@
         <v>289</v>
       </c>
       <c r="C99" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D99" t="s">
         <v>290</v>
@@ -4431,7 +4443,7 @@
         <v>295</v>
       </c>
       <c r="C101" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D101" t="s">
         <v>296</v>
@@ -4448,7 +4460,7 @@
         <v>298</v>
       </c>
       <c r="C102" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D102" t="s">
         <v>299</v>
@@ -4465,7 +4477,7 @@
         <v>301</v>
       </c>
       <c r="C103" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D103" t="s">
         <v>302</v>
@@ -4482,7 +4494,7 @@
         <v>304</v>
       </c>
       <c r="C104" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D104" t="s">
         <v>305</v>
@@ -4499,7 +4511,7 @@
         <v>307</v>
       </c>
       <c r="C105" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D105" t="s">
         <v>308</v>
@@ -4516,7 +4528,7 @@
         <v>310</v>
       </c>
       <c r="C106" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D106" t="s">
         <v>311</v>
@@ -4533,7 +4545,7 @@
         <v>313</v>
       </c>
       <c r="C107" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D107" t="s">
         <v>314</v>
@@ -4567,13 +4579,13 @@
         <v>319</v>
       </c>
       <c r="C109" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D109" t="s">
         <v>320</v>
       </c>
       <c r="E109" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
@@ -4584,13 +4596,13 @@
         <v>321</v>
       </c>
       <c r="C110" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D110" t="s">
         <v>322</v>
       </c>
       <c r="E110" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
@@ -4601,13 +4613,13 @@
         <v>323</v>
       </c>
       <c r="C111" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D111" t="s">
         <v>324</v>
       </c>
       <c r="E111" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
@@ -4618,13 +4630,13 @@
         <v>325</v>
       </c>
       <c r="C112" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D112" t="s">
         <v>326</v>
       </c>
       <c r="E112" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
@@ -4635,13 +4647,13 @@
         <v>327</v>
       </c>
       <c r="C113" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D113" t="s">
         <v>328</v>
       </c>
       <c r="E113" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
@@ -4658,7 +4670,7 @@
         <v>330</v>
       </c>
       <c r="E114" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
@@ -4669,7 +4681,7 @@
         <v>331</v>
       </c>
       <c r="C115" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D115" t="s">
         <v>332</v>
@@ -4686,13 +4698,13 @@
         <v>334</v>
       </c>
       <c r="C116" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D116" t="s">
         <v>335</v>
       </c>
       <c r="E116" t="s">
-        <v>735</v>
+        <v>727</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
@@ -4703,13 +4715,13 @@
         <v>336</v>
       </c>
       <c r="C117" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D117" t="s">
         <v>337</v>
       </c>
       <c r="E117" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
@@ -4737,7 +4749,7 @@
         <v>341</v>
       </c>
       <c r="C119" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D119" t="s">
         <v>342</v>
@@ -4771,7 +4783,7 @@
         <v>347</v>
       </c>
       <c r="C121" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D121" t="s">
         <v>348</v>
@@ -4788,7 +4800,7 @@
         <v>350</v>
       </c>
       <c r="C122" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D122" t="s">
         <v>351</v>
@@ -4822,7 +4834,7 @@
         <v>356</v>
       </c>
       <c r="C124" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D124" t="s">
         <v>357</v>
@@ -4839,7 +4851,7 @@
         <v>359</v>
       </c>
       <c r="C125" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D125" t="s">
         <v>360</v>
@@ -4856,7 +4868,7 @@
         <v>362</v>
       </c>
       <c r="C126" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D126" t="s">
         <v>363</v>
@@ -4873,7 +4885,7 @@
         <v>365</v>
       </c>
       <c r="C127" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D127" t="s">
         <v>366</v>
@@ -4890,7 +4902,7 @@
         <v>368</v>
       </c>
       <c r="C128" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D128" t="s">
         <v>369</v>
@@ -4907,7 +4919,7 @@
         <v>371</v>
       </c>
       <c r="C129" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D129" t="s">
         <v>372</v>
@@ -4930,7 +4942,7 @@
         <v>375</v>
       </c>
       <c r="E130" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
@@ -4941,7 +4953,7 @@
         <v>376</v>
       </c>
       <c r="C131" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D131" t="s">
         <v>377</v>
@@ -4958,7 +4970,7 @@
         <v>379</v>
       </c>
       <c r="C132" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D132" t="s">
         <v>380</v>
@@ -4975,7 +4987,7 @@
         <v>382</v>
       </c>
       <c r="C133" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D133" t="s">
         <v>383</v>
@@ -4992,7 +5004,7 @@
         <v>385</v>
       </c>
       <c r="C134" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D134" t="s">
         <v>386</v>
@@ -5009,7 +5021,7 @@
         <v>388</v>
       </c>
       <c r="C135" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D135" t="s">
         <v>389</v>
@@ -5026,7 +5038,7 @@
         <v>391</v>
       </c>
       <c r="C136" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D136" t="s">
         <v>392</v>
@@ -5060,7 +5072,7 @@
         <v>397</v>
       </c>
       <c r="C138" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D138" t="s">
         <v>398</v>
@@ -5077,7 +5089,7 @@
         <v>400</v>
       </c>
       <c r="C139" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D139" t="s">
         <v>401</v>
@@ -5100,7 +5112,7 @@
         <v>404</v>
       </c>
       <c r="E140" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
@@ -5111,13 +5123,13 @@
         <v>405</v>
       </c>
       <c r="C141" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D141" t="s">
         <v>406</v>
       </c>
       <c r="E141" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
@@ -5145,7 +5157,7 @@
         <v>409</v>
       </c>
       <c r="C143" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D143" t="s">
         <v>410</v>
@@ -5179,13 +5191,13 @@
         <v>415</v>
       </c>
       <c r="C145" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D145" t="s">
         <v>416</v>
       </c>
       <c r="E145" t="s">
-        <v>740</v>
+        <v>732</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
@@ -5196,7 +5208,7 @@
         <v>417</v>
       </c>
       <c r="C146" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D146" t="s">
         <v>418</v>
@@ -5213,7 +5225,7 @@
         <v>420</v>
       </c>
       <c r="C147" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D147" t="s">
         <v>421</v>
@@ -5230,7 +5242,7 @@
         <v>423</v>
       </c>
       <c r="C148" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D148" t="s">
         <v>424</v>
@@ -5247,7 +5259,7 @@
         <v>426</v>
       </c>
       <c r="C149" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D149" t="s">
         <v>427</v>
@@ -5264,7 +5276,7 @@
         <v>429</v>
       </c>
       <c r="C150" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D150" t="s">
         <v>430</v>
@@ -5281,7 +5293,7 @@
         <v>432</v>
       </c>
       <c r="C151" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D151" t="s">
         <v>433</v>
@@ -5298,7 +5310,7 @@
         <v>435</v>
       </c>
       <c r="C152" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D152" t="s">
         <v>436</v>
@@ -5315,7 +5327,7 @@
         <v>438</v>
       </c>
       <c r="C153" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D153" t="s">
         <v>439</v>
@@ -5332,7 +5344,7 @@
         <v>441</v>
       </c>
       <c r="C154" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D154" t="s">
         <v>442</v>
@@ -5349,7 +5361,7 @@
         <v>444</v>
       </c>
       <c r="C155" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D155" t="s">
         <v>445</v>
@@ -5366,13 +5378,13 @@
         <v>447</v>
       </c>
       <c r="C156" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D156" t="s">
         <v>448</v>
       </c>
       <c r="E156" t="s">
-        <v>741</v>
+        <v>733</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
@@ -5400,13 +5412,13 @@
         <v>452</v>
       </c>
       <c r="C158" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D158" t="s">
         <v>453</v>
       </c>
       <c r="E158" t="s">
-        <v>742</v>
+        <v>734</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
@@ -5417,13 +5429,13 @@
         <v>454</v>
       </c>
       <c r="C159" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D159" t="s">
         <v>455</v>
       </c>
       <c r="E159" t="s">
-        <v>743</v>
+        <v>735</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
@@ -5434,13 +5446,13 @@
         <v>456</v>
       </c>
       <c r="C160" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D160" t="s">
         <v>457</v>
       </c>
       <c r="E160" t="s">
-        <v>744</v>
+        <v>736</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
@@ -5451,13 +5463,13 @@
         <v>458</v>
       </c>
       <c r="C161" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D161" t="s">
         <v>459</v>
       </c>
       <c r="E161" t="s">
-        <v>745</v>
+        <v>737</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
@@ -5468,13 +5480,13 @@
         <v>460</v>
       </c>
       <c r="C162" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D162" t="s">
         <v>461</v>
       </c>
       <c r="E162" t="s">
-        <v>746</v>
+        <v>738</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
@@ -5485,13 +5497,13 @@
         <v>462</v>
       </c>
       <c r="C163" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D163" t="s">
         <v>463</v>
       </c>
       <c r="E163" t="s">
-        <v>747</v>
+        <v>739</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
@@ -5502,13 +5514,13 @@
         <v>464</v>
       </c>
       <c r="C164" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D164" t="s">
         <v>465</v>
       </c>
       <c r="E164" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
@@ -5519,13 +5531,13 @@
         <v>466</v>
       </c>
       <c r="C165" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D165" t="s">
         <v>467</v>
       </c>
       <c r="E165" t="s">
-        <v>749</v>
+        <v>741</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
@@ -5536,13 +5548,13 @@
         <v>468</v>
       </c>
       <c r="C166" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D166" t="s">
         <v>469</v>
       </c>
       <c r="E166" t="s">
-        <v>750</v>
+        <v>742</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
@@ -5570,7 +5582,7 @@
         <v>473</v>
       </c>
       <c r="C168" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D168" t="s">
         <v>474</v>
@@ -5587,7 +5599,7 @@
         <v>476</v>
       </c>
       <c r="C169" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D169" t="s">
         <v>477</v>
@@ -5604,13 +5616,13 @@
         <v>479</v>
       </c>
       <c r="C170" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D170" t="s">
         <v>480</v>
       </c>
       <c r="E170" t="s">
-        <v>751</v>
+        <v>743</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
@@ -5621,13 +5633,13 @@
         <v>481</v>
       </c>
       <c r="C171" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D171" t="s">
         <v>482</v>
       </c>
       <c r="E171" t="s">
-        <v>752</v>
+        <v>744</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
@@ -5638,13 +5650,13 @@
         <v>483</v>
       </c>
       <c r="C172" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D172" t="s">
         <v>484</v>
       </c>
       <c r="E172" t="s">
-        <v>753</v>
+        <v>745</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
@@ -5655,13 +5667,13 @@
         <v>485</v>
       </c>
       <c r="C173" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D173" t="s">
         <v>486</v>
       </c>
       <c r="E173" t="s">
-        <v>754</v>
+        <v>746</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
@@ -5672,13 +5684,13 @@
         <v>487</v>
       </c>
       <c r="C174" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D174" t="s">
         <v>488</v>
       </c>
       <c r="E174" t="s">
-        <v>755</v>
+        <v>747</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
@@ -5689,13 +5701,13 @@
         <v>489</v>
       </c>
       <c r="C175" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D175" t="s">
         <v>490</v>
       </c>
       <c r="E175" t="s">
-        <v>756</v>
+        <v>748</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
@@ -5706,13 +5718,13 @@
         <v>491</v>
       </c>
       <c r="C176" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D176" t="s">
         <v>492</v>
       </c>
       <c r="E176" t="s">
-        <v>757</v>
+        <v>749</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
@@ -5723,13 +5735,13 @@
         <v>493</v>
       </c>
       <c r="C177" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D177" t="s">
         <v>494</v>
       </c>
       <c r="E177" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
@@ -5740,13 +5752,13 @@
         <v>495</v>
       </c>
       <c r="C178" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D178" t="s">
         <v>496</v>
       </c>
       <c r="E178" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
@@ -5774,7 +5786,7 @@
         <v>500</v>
       </c>
       <c r="C180" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D180" t="s">
         <v>501</v>
@@ -5791,7 +5803,7 @@
         <v>503</v>
       </c>
       <c r="C181" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D181" t="s">
         <v>504</v>
@@ -5808,13 +5820,13 @@
         <v>506</v>
       </c>
       <c r="C182" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D182" t="s">
         <v>507</v>
       </c>
       <c r="E182" t="s">
-        <v>760</v>
+        <v>752</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
@@ -5825,13 +5837,13 @@
         <v>508</v>
       </c>
       <c r="C183" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D183" t="s">
         <v>509</v>
       </c>
       <c r="E183" t="s">
-        <v>761</v>
+        <v>753</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
@@ -5842,13 +5854,13 @@
         <v>510</v>
       </c>
       <c r="C184" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D184" t="s">
         <v>511</v>
       </c>
       <c r="E184" t="s">
-        <v>762</v>
+        <v>754</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
@@ -5859,13 +5871,13 @@
         <v>512</v>
       </c>
       <c r="C185" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D185" t="s">
         <v>513</v>
       </c>
       <c r="E185" t="s">
-        <v>763</v>
+        <v>755</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
@@ -5876,13 +5888,13 @@
         <v>514</v>
       </c>
       <c r="C186" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D186" t="s">
         <v>515</v>
       </c>
       <c r="E186" t="s">
-        <v>764</v>
+        <v>756</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.3">
@@ -5893,13 +5905,13 @@
         <v>516</v>
       </c>
       <c r="C187" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D187" t="s">
         <v>517</v>
       </c>
       <c r="E187" t="s">
-        <v>765</v>
+        <v>757</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
@@ -5910,13 +5922,13 @@
         <v>518</v>
       </c>
       <c r="C188" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D188" t="s">
         <v>519</v>
       </c>
       <c r="E188" t="s">
-        <v>766</v>
+        <v>758</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
@@ -5944,7 +5956,7 @@
         <v>522</v>
       </c>
       <c r="C190" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D190" t="s">
         <v>523</v>
@@ -5978,7 +5990,7 @@
         <v>528</v>
       </c>
       <c r="C192" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D192" t="s">
         <v>529</v>
@@ -5995,7 +6007,7 @@
         <v>531</v>
       </c>
       <c r="C193" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D193" t="s">
         <v>532</v>
@@ -6012,7 +6024,7 @@
         <v>534</v>
       </c>
       <c r="C194" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D194" t="s">
         <v>535</v>
@@ -6046,7 +6058,7 @@
         <v>540</v>
       </c>
       <c r="C196" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D196" t="s">
         <v>541</v>
@@ -6063,7 +6075,7 @@
         <v>543</v>
       </c>
       <c r="C197" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D197" t="s">
         <v>544</v>
@@ -6080,7 +6092,7 @@
         <v>546</v>
       </c>
       <c r="C198" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D198" t="s">
         <v>547</v>
@@ -6097,7 +6109,7 @@
         <v>549</v>
       </c>
       <c r="C199" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D199" t="s">
         <v>550</v>
@@ -6114,7 +6126,7 @@
         <v>552</v>
       </c>
       <c r="C200" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D200" t="s">
         <v>553</v>
@@ -6131,7 +6143,7 @@
         <v>555</v>
       </c>
       <c r="C201" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D201" t="s">
         <v>556</v>
@@ -6148,7 +6160,7 @@
         <v>558</v>
       </c>
       <c r="C202" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D202" t="s">
         <v>559</v>
@@ -6165,7 +6177,7 @@
         <v>561</v>
       </c>
       <c r="C203" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D203" t="s">
         <v>562</v>
@@ -6182,7 +6194,7 @@
         <v>564</v>
       </c>
       <c r="C204" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D204" t="s">
         <v>565</v>
@@ -6199,7 +6211,7 @@
         <v>567</v>
       </c>
       <c r="C205" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D205" t="s">
         <v>568</v>
@@ -6222,7 +6234,7 @@
         <v>571</v>
       </c>
       <c r="E206" t="s">
-        <v>572</v>
+        <v>777</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.3">
@@ -6230,16 +6242,16 @@
         <v>206</v>
       </c>
       <c r="B207" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C207" t="s">
         <v>11</v>
       </c>
       <c r="D207" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E207" t="s">
-        <v>575</v>
+        <v>778</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.3">
@@ -6247,16 +6259,16 @@
         <v>207</v>
       </c>
       <c r="B208" t="s">
+        <v>574</v>
+      </c>
+      <c r="C208" t="s">
+        <v>772</v>
+      </c>
+      <c r="D208" t="s">
+        <v>575</v>
+      </c>
+      <c r="E208" t="s">
         <v>576</v>
-      </c>
-      <c r="C208" t="s">
-        <v>54</v>
-      </c>
-      <c r="D208" t="s">
-        <v>577</v>
-      </c>
-      <c r="E208" t="s">
-        <v>578</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.3">
@@ -6264,16 +6276,16 @@
         <v>208</v>
       </c>
       <c r="B209" t="s">
+        <v>577</v>
+      </c>
+      <c r="C209" t="s">
+        <v>772</v>
+      </c>
+      <c r="D209" t="s">
+        <v>578</v>
+      </c>
+      <c r="E209" t="s">
         <v>579</v>
-      </c>
-      <c r="C209" t="s">
-        <v>54</v>
-      </c>
-      <c r="D209" t="s">
-        <v>580</v>
-      </c>
-      <c r="E209" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.3">
@@ -6281,16 +6293,16 @@
         <v>209</v>
       </c>
       <c r="B210" t="s">
+        <v>580</v>
+      </c>
+      <c r="C210" t="s">
+        <v>772</v>
+      </c>
+      <c r="D210" t="s">
+        <v>581</v>
+      </c>
+      <c r="E210" t="s">
         <v>582</v>
-      </c>
-      <c r="C210" t="s">
-        <v>54</v>
-      </c>
-      <c r="D210" t="s">
-        <v>583</v>
-      </c>
-      <c r="E210" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
@@ -6298,16 +6310,16 @@
         <v>210</v>
       </c>
       <c r="B211" t="s">
+        <v>583</v>
+      </c>
+      <c r="C211" t="s">
+        <v>772</v>
+      </c>
+      <c r="D211" t="s">
+        <v>584</v>
+      </c>
+      <c r="E211" t="s">
         <v>585</v>
-      </c>
-      <c r="C211" t="s">
-        <v>54</v>
-      </c>
-      <c r="D211" t="s">
-        <v>586</v>
-      </c>
-      <c r="E211" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
@@ -6315,16 +6327,16 @@
         <v>211</v>
       </c>
       <c r="B212" t="s">
+        <v>586</v>
+      </c>
+      <c r="C212" t="s">
+        <v>772</v>
+      </c>
+      <c r="D212" t="s">
+        <v>587</v>
+      </c>
+      <c r="E212" t="s">
         <v>588</v>
-      </c>
-      <c r="C212" t="s">
-        <v>54</v>
-      </c>
-      <c r="D212" t="s">
-        <v>589</v>
-      </c>
-      <c r="E212" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
@@ -6332,16 +6344,16 @@
         <v>212</v>
       </c>
       <c r="B213" t="s">
+        <v>589</v>
+      </c>
+      <c r="C213" t="s">
+        <v>772</v>
+      </c>
+      <c r="D213" t="s">
+        <v>590</v>
+      </c>
+      <c r="E213" t="s">
         <v>591</v>
-      </c>
-      <c r="C213" t="s">
-        <v>54</v>
-      </c>
-      <c r="D213" t="s">
-        <v>592</v>
-      </c>
-      <c r="E213" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.3">
@@ -6349,16 +6361,16 @@
         <v>213</v>
       </c>
       <c r="B214" t="s">
+        <v>592</v>
+      </c>
+      <c r="C214" t="s">
+        <v>772</v>
+      </c>
+      <c r="D214" t="s">
+        <v>593</v>
+      </c>
+      <c r="E214" t="s">
         <v>594</v>
-      </c>
-      <c r="C214" t="s">
-        <v>54</v>
-      </c>
-      <c r="D214" t="s">
-        <v>595</v>
-      </c>
-      <c r="E214" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.3">
@@ -6366,13 +6378,13 @@
         <v>214</v>
       </c>
       <c r="B215" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C215" t="s">
         <v>11</v>
       </c>
       <c r="D215" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="E215" t="s">
         <v>340</v>
@@ -6383,16 +6395,16 @@
         <v>215</v>
       </c>
       <c r="B216" t="s">
+        <v>597</v>
+      </c>
+      <c r="C216" t="s">
+        <v>772</v>
+      </c>
+      <c r="D216" t="s">
+        <v>598</v>
+      </c>
+      <c r="E216" t="s">
         <v>599</v>
-      </c>
-      <c r="C216" t="s">
-        <v>11</v>
-      </c>
-      <c r="D216" t="s">
-        <v>600</v>
-      </c>
-      <c r="E216" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.3">
@@ -6400,16 +6412,16 @@
         <v>216</v>
       </c>
       <c r="B217" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C217" t="s">
         <v>11</v>
       </c>
       <c r="D217" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E217" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.3">
@@ -6417,16 +6429,16 @@
         <v>217</v>
       </c>
       <c r="B218" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C218" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D218" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="E218" t="s">
-        <v>767</v>
+        <v>759</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.3">
@@ -6434,16 +6446,16 @@
         <v>218</v>
       </c>
       <c r="B219" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C219" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D219" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E219" t="s">
-        <v>768</v>
+        <v>760</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.3">
@@ -6451,16 +6463,16 @@
         <v>219</v>
       </c>
       <c r="B220" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="C220" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D220" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E220" t="s">
-        <v>769</v>
+        <v>761</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.3">
@@ -6468,16 +6480,16 @@
         <v>220</v>
       </c>
       <c r="B221" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="C221" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D221" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E221" t="s">
-        <v>770</v>
+        <v>762</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.3">
@@ -6485,16 +6497,16 @@
         <v>221</v>
       </c>
       <c r="B222" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="C222" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D222" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="E222" t="s">
-        <v>771</v>
+        <v>763</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.3">
@@ -6502,16 +6514,16 @@
         <v>222</v>
       </c>
       <c r="B223" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="C223" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D223" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E223" t="s">
-        <v>772</v>
+        <v>764</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.3">
@@ -6519,16 +6531,16 @@
         <v>223</v>
       </c>
       <c r="B224" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="C224" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D224" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E224" t="s">
-        <v>773</v>
+        <v>765</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.3">
@@ -6536,16 +6548,16 @@
         <v>224</v>
       </c>
       <c r="B225" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C225" t="s">
         <v>11</v>
       </c>
       <c r="D225" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E225" t="s">
-        <v>774</v>
+        <v>766</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.3">
@@ -6553,16 +6565,16 @@
         <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="C226" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D226" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="E226" t="s">
-        <v>623</v>
+        <v>779</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.3">
@@ -6570,16 +6582,16 @@
         <v>226</v>
       </c>
       <c r="B227" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C227" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D227" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="E227" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.3">
@@ -6587,16 +6599,16 @@
         <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="C228" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D228" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="E228" t="s">
-        <v>629</v>
+        <v>780</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.3">
@@ -6604,16 +6616,16 @@
         <v>228</v>
       </c>
       <c r="B229" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C229" t="s">
         <v>11</v>
       </c>
       <c r="D229" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="E229" t="s">
-        <v>632</v>
+        <v>781</v>
       </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.3">
@@ -6621,16 +6633,16 @@
         <v>229</v>
       </c>
       <c r="B230" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="C230" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D230" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="E230" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.3">
@@ -6638,16 +6650,16 @@
         <v>230</v>
       </c>
       <c r="B231" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="C231" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D231" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="E231" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.3">
@@ -6655,16 +6667,16 @@
         <v>231</v>
       </c>
       <c r="B232" t="s">
-        <v>639</v>
+        <v>634</v>
       </c>
       <c r="C232" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D232" t="s">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="E232" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.3">
@@ -6672,16 +6684,16 @@
         <v>232</v>
       </c>
       <c r="B233" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="C233" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D233" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="E233" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.3">
@@ -6689,16 +6701,16 @@
         <v>233</v>
       </c>
       <c r="B234" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="C234" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D234" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="E234" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.3">
@@ -6706,16 +6718,16 @@
         <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="C235" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D235" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="E235" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.3">
@@ -6723,16 +6735,16 @@
         <v>235</v>
       </c>
       <c r="B236" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="C236" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D236" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="E236" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.3">
@@ -6740,16 +6752,16 @@
         <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="C237" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D237" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="E237" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.3">
@@ -6757,16 +6769,16 @@
         <v>237</v>
       </c>
       <c r="B238" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="C238" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D238" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="E238" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.3">
@@ -6774,16 +6786,16 @@
         <v>238</v>
       </c>
       <c r="B239" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="C239" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D239" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
       <c r="E239" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.3">
@@ -6791,16 +6803,16 @@
         <v>239</v>
       </c>
       <c r="B240" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="C240" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D240" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
       <c r="E240" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.3">
@@ -6808,16 +6820,16 @@
         <v>240</v>
       </c>
       <c r="B241" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="C241" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D241" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="E241" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.3">
@@ -6825,16 +6837,16 @@
         <v>241</v>
       </c>
       <c r="B242" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="C242" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="D242" t="s">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="E242" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.3">
@@ -6842,13 +6854,13 @@
         <v>242</v>
       </c>
       <c r="B243" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="C243" t="s">
         <v>11</v>
       </c>
       <c r="D243" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="E243" t="s">
         <v>340</v>
@@ -6859,16 +6871,16 @@
         <v>243</v>
       </c>
       <c r="B244" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="C244" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D244" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
       <c r="E244" t="s">
-        <v>676</v>
+        <v>774</v>
       </c>
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.3">
@@ -6876,16 +6888,16 @@
         <v>244</v>
       </c>
       <c r="B245" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="C245" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D245" t="s">
-        <v>678</v>
+        <v>672</v>
       </c>
       <c r="E245" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.3">
@@ -6893,16 +6905,16 @@
         <v>245</v>
       </c>
       <c r="B246" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
       <c r="C246" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D246" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="E246" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
     </row>
     <row r="247" spans="1:5" x14ac:dyDescent="0.3">
@@ -6910,16 +6922,16 @@
         <v>246</v>
       </c>
       <c r="B247" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="C247" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D247" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
       <c r="E247" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.3">
@@ -6927,16 +6939,16 @@
         <v>247</v>
       </c>
       <c r="B248" t="s">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="C248" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D248" t="s">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="E248" t="s">
-        <v>688</v>
+        <v>682</v>
       </c>
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.3">
@@ -6944,16 +6956,16 @@
         <v>248</v>
       </c>
       <c r="B249" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
       <c r="C249" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D249" t="s">
-        <v>690</v>
+        <v>684</v>
       </c>
       <c r="E249" t="s">
-        <v>691</v>
+        <v>685</v>
       </c>
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.3">
@@ -6961,16 +6973,16 @@
         <v>249</v>
       </c>
       <c r="B250" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="C250" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D250" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="E250" t="s">
-        <v>694</v>
+        <v>688</v>
       </c>
     </row>
     <row r="251" spans="1:5" x14ac:dyDescent="0.3">
@@ -6978,16 +6990,16 @@
         <v>250</v>
       </c>
       <c r="B251" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="C251" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D251" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="E251" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.3">
@@ -6995,16 +7007,16 @@
         <v>251</v>
       </c>
       <c r="B252" t="s">
-        <v>698</v>
+        <v>692</v>
       </c>
       <c r="C252" t="s">
         <v>54</v>
       </c>
       <c r="D252" t="s">
-        <v>699</v>
+        <v>693</v>
       </c>
       <c r="E252" t="s">
-        <v>700</v>
+        <v>782</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.3">
@@ -7012,16 +7024,16 @@
         <v>252</v>
       </c>
       <c r="B253" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="C253" t="s">
         <v>54</v>
       </c>
       <c r="D253" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
       <c r="E253" t="s">
-        <v>703</v>
+        <v>783</v>
       </c>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.3">
@@ -7029,16 +7041,16 @@
         <v>253</v>
       </c>
       <c r="B254" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="C254" t="s">
-        <v>11</v>
+        <v>772</v>
       </c>
       <c r="D254" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="E254" t="s">
-        <v>705</v>
+        <v>784</v>
       </c>
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.3">
@@ -7046,16 +7058,16 @@
         <v>254</v>
       </c>
       <c r="B255" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="C255" t="s">
         <v>11</v>
       </c>
       <c r="D255" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="E255" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.3">
@@ -7063,16 +7075,16 @@
         <v>255</v>
       </c>
       <c r="B256" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="C256" t="s">
         <v>11</v>
       </c>
       <c r="D256" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="E256" t="s">
-        <v>775</v>
+        <v>767</v>
       </c>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.3">
@@ -7080,16 +7092,16 @@
         <v>256</v>
       </c>
       <c r="B257" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="C257" t="s">
         <v>54</v>
       </c>
       <c r="D257" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="E257" t="s">
-        <v>776</v>
+        <v>768</v>
       </c>
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.3">
@@ -7097,16 +7109,16 @@
         <v>257</v>
       </c>
       <c r="B258" t="s">
-        <v>712</v>
+        <v>704</v>
       </c>
       <c r="C258" t="s">
         <v>54</v>
       </c>
       <c r="D258" t="s">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="E258" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.3">
@@ -7114,16 +7126,16 @@
         <v>258</v>
       </c>
       <c r="B259" t="s">
-        <v>714</v>
+        <v>706</v>
       </c>
       <c r="C259" t="s">
         <v>54</v>
       </c>
       <c r="D259" t="s">
-        <v>715</v>
+        <v>707</v>
       </c>
       <c r="E259" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.3">
@@ -7131,16 +7143,16 @@
         <v>259</v>
       </c>
       <c r="B260" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="C260" t="s">
         <v>54</v>
       </c>
       <c r="D260" t="s">
-        <v>717</v>
+        <v>709</v>
       </c>
       <c r="E260" t="s">
-        <v>779</v>
+        <v>771</v>
       </c>
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.3">
@@ -7148,16 +7160,16 @@
         <v>260</v>
       </c>
       <c r="B261" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="C261" t="s">
         <v>54</v>
       </c>
       <c r="D261" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="E261" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.3">
@@ -7165,16 +7177,16 @@
         <v>261</v>
       </c>
       <c r="B262" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="C262" t="s">
         <v>11</v>
       </c>
       <c r="D262" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="E262" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.3">
@@ -7182,16 +7194,16 @@
         <v>262</v>
       </c>
       <c r="B263" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
       <c r="C263" t="s">
         <v>6</v>
       </c>
       <c r="D263" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
       <c r="E263" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.3">
@@ -7199,16 +7211,16 @@
         <v>263</v>
       </c>
       <c r="B264" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
       <c r="C264" t="s">
         <v>11</v>
       </c>
       <c r="D264" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
       <c r="E264" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.3">
@@ -7216,16 +7228,16 @@
         <v>264</v>
       </c>
       <c r="B265" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
       <c r="C265" t="s">
         <v>11</v>
       </c>
       <c r="D265" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
       <c r="E265" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.3">
@@ -7233,16 +7245,16 @@
         <v>265</v>
       </c>
       <c r="B266" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="C266" t="s">
         <v>11</v>
       </c>
       <c r="D266" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="E266" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.3">
@@ -7250,16 +7262,16 @@
         <v>266</v>
       </c>
       <c r="B267" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="C267" t="s">
         <v>54</v>
       </c>
       <c r="D267" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="E267" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>